<commit_message>
WIP (BLOCKED — DO NOT MERGE): Dumbbell Pullovers, load classification unresolved
Everything authored and verified except load. No existing load category fits:
PREHAB_NO_LOAD returns the right null but makes the card render "BW" for a
dumbbell exercise (isTrueBodyweightExercise covers both sets, and formatWeight
keys the label off it). EXERCISE_LOAD_MAP requires anchor+ratio, which would
prescribe a weight Sam ruled athlete-chosen. Unlisted invents 12.5kg.

Awaiting Sam's ruling on a third typed set (ATHLETE_CHOSEN_LOAD_EXERCISES).
Committed only so the work is not lost. Gates would pass — that is the point:
the content lock cannot see a UI label.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/MUSCLE_EXPERIENCE_FINAL_2026-07-25.xlsx
+++ b/docs/MUSCLE_EXPERIENCE_FINAL_2026-07-25.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F203"/>
+  <dimension ref="A1:F204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4688,17 +4688,17 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>Easy cardio (zone 1)</t>
+          <t>Mobility</t>
         </is>
       </c>
       <c r="B151" s="1" t="inlineStr">
         <is>
-          <t>Light Walk or Stationary Bike</t>
+          <t>Dumbbell Pullovers</t>
         </is>
       </c>
       <c r="C151" s="1" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Upper back, Shoulders</t>
         </is>
       </c>
       <c r="D151" s="1" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="B152" s="1" t="inlineStr">
         <is>
-          <t>Incline Treadmill Walk</t>
+          <t>Light Walk or Stationary Bike</t>
         </is>
       </c>
       <c r="C152" s="1" t="inlineStr">
@@ -4749,7 +4749,7 @@
       </c>
       <c r="B153" s="1" t="inlineStr">
         <is>
-          <t>Outdoor Walk</t>
+          <t>Incline Treadmill Walk</t>
         </is>
       </c>
       <c r="C153" s="1" t="inlineStr">
@@ -4777,12 +4777,12 @@
       </c>
       <c r="B154" s="1" t="inlineStr">
         <is>
-          <t>Light Skipping</t>
+          <t>Outdoor Walk</t>
         </is>
       </c>
       <c r="C154" s="1" t="inlineStr">
         <is>
-          <t>Calves</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D154" s="1" t="inlineStr">
@@ -4800,17 +4800,17 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>Breathing reset</t>
+          <t>Easy cardio (zone 1)</t>
         </is>
       </c>
       <c r="B155" s="1" t="inlineStr">
         <is>
-          <t>90/90 Breathing</t>
+          <t>Light Skipping</t>
         </is>
       </c>
       <c r="C155" s="1" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Calves</t>
         </is>
       </c>
       <c r="D155" s="1" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="B156" s="1" t="inlineStr">
         <is>
-          <t>Crocodile Breathing</t>
+          <t>90/90 Breathing</t>
         </is>
       </c>
       <c r="C156" s="1" t="inlineStr">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="B157" s="1" t="inlineStr">
         <is>
-          <t>Box Breathing</t>
+          <t>Crocodile Breathing</t>
         </is>
       </c>
       <c r="C157" s="1" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="B158" s="1" t="inlineStr">
         <is>
-          <t>Child's Pose with Breathing</t>
+          <t>Box Breathing</t>
         </is>
       </c>
       <c r="C158" s="1" t="inlineStr">
@@ -4912,12 +4912,12 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>Conditioning</t>
+          <t>Breathing reset</t>
         </is>
       </c>
       <c r="B159" s="1" t="inlineStr">
         <is>
-          <t>Sprint Intervals</t>
+          <t>Child's Pose with Breathing</t>
         </is>
       </c>
       <c r="C159" s="1" t="inlineStr">
@@ -4932,14 +4932,10 @@
       </c>
       <c r="E159" s="1" t="inlineStr">
         <is>
-          <t>1+ years</t>
-        </is>
-      </c>
-      <c r="F159" s="1" t="inlineStr">
-        <is>
-          <t>⚑ field sprint at top-end speed; hamstring/calf tagged 'avoid'. Gate here is conditioning base, not lifting experience, so this ladder may not be the right instrument at all.</t>
-        </is>
-      </c>
+          <t>everyone</t>
+        </is>
+      </c>
+      <c r="F159" s="1" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="1" t="inlineStr">
@@ -4949,7 +4945,7 @@
       </c>
       <c r="B160" s="1" t="inlineStr">
         <is>
-          <t>Hill Sprints</t>
+          <t>Sprint Intervals</t>
         </is>
       </c>
       <c r="C160" s="1" t="inlineStr">
@@ -4981,7 +4977,7 @@
       </c>
       <c r="B161" s="1" t="inlineStr">
         <is>
-          <t>Quality Sprints</t>
+          <t>Hill Sprints</t>
         </is>
       </c>
       <c r="C161" s="1" t="inlineStr">
@@ -5013,7 +5009,7 @@
       </c>
       <c r="B162" s="1" t="inlineStr">
         <is>
-          <t>MAS Training</t>
+          <t>Quality Sprints</t>
         </is>
       </c>
       <c r="C162" s="1" t="inlineStr">
@@ -5045,7 +5041,7 @@
       </c>
       <c r="B163" s="1" t="inlineStr">
         <is>
-          <t>Flying Sprints</t>
+          <t>MAS Training</t>
         </is>
       </c>
       <c r="C163" s="1" t="inlineStr">
@@ -5065,7 +5061,7 @@
       </c>
       <c r="F163" s="1" t="inlineStr">
         <is>
-          <t>⚑ field sprint at top-end speed. Gate here is conditioning base, not lifting experience, so this ladder may not be the right instrument at all.</t>
+          <t>⚑ field sprint at top-end speed; hamstring/calf tagged 'avoid'. Gate here is conditioning base, not lifting experience, so this ladder may not be the right instrument at all.</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5073,7 @@
       </c>
       <c r="B164" s="1" t="inlineStr">
         <is>
-          <t>MAS 15:15 Blocks</t>
+          <t>Flying Sprints</t>
         </is>
       </c>
       <c r="C164" s="1" t="inlineStr">
@@ -5109,7 +5105,7 @@
       </c>
       <c r="B165" s="1" t="inlineStr">
         <is>
-          <t>Tabata Intervals</t>
+          <t>MAS 15:15 Blocks</t>
         </is>
       </c>
       <c r="C165" s="1" t="inlineStr">
@@ -5124,12 +5120,12 @@
       </c>
       <c r="E165" s="1" t="inlineStr">
         <is>
-          <t>everyone</t>
+          <t>1+ years</t>
         </is>
       </c>
       <c r="F165" s="1" t="inlineStr">
         <is>
-          <t>session format, not an individual movement — no meaningful muscle group.</t>
+          <t>⚑ field sprint at top-end speed. Gate here is conditioning base, not lifting experience, so this ladder may not be the right instrument at all.</t>
         </is>
       </c>
     </row>
@@ -5141,7 +5137,7 @@
       </c>
       <c r="B166" s="1" t="inlineStr">
         <is>
-          <t>Inverse Tabata</t>
+          <t>Tabata Intervals</t>
         </is>
       </c>
       <c r="C166" s="1" t="inlineStr">
@@ -5173,7 +5169,7 @@
       </c>
       <c r="B167" s="1" t="inlineStr">
         <is>
-          <t>Max Effort Sprint Accumulation</t>
+          <t>Inverse Tabata</t>
         </is>
       </c>
       <c r="C167" s="1" t="inlineStr">
@@ -5205,7 +5201,7 @@
       </c>
       <c r="B168" s="1" t="inlineStr">
         <is>
-          <t>Free Sprint Session</t>
+          <t>Max Effort Sprint Accumulation</t>
         </is>
       </c>
       <c r="C168" s="1" t="inlineStr">
@@ -5220,12 +5216,12 @@
       </c>
       <c r="E168" s="1" t="inlineStr">
         <is>
-          <t>1+ years</t>
+          <t>everyone</t>
         </is>
       </c>
       <c r="F168" s="1" t="inlineStr">
         <is>
-          <t>⚑ field sprint at top-end speed; hamstring/calf tagged 'avoid'. Gate here is conditioning base, not lifting experience, so this ladder may not be the right instrument at all.</t>
+          <t>session format, not an individual movement — no meaningful muscle group.</t>
         </is>
       </c>
     </row>
@@ -5237,7 +5233,7 @@
       </c>
       <c r="B169" s="1" t="inlineStr">
         <is>
-          <t>Long Run</t>
+          <t>Free Sprint Session</t>
         </is>
       </c>
       <c r="C169" s="1" t="inlineStr">
@@ -5252,12 +5248,12 @@
       </c>
       <c r="E169" s="1" t="inlineStr">
         <is>
-          <t>everyone</t>
+          <t>1+ years</t>
         </is>
       </c>
       <c r="F169" s="1" t="inlineStr">
         <is>
-          <t>session format, not an individual movement — no meaningful muscle group.</t>
+          <t>⚑ field sprint at top-end speed; hamstring/calf tagged 'avoid'. Gate here is conditioning base, not lifting experience, so this ladder may not be the right instrument at all.</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5265,7 @@
       </c>
       <c r="B170" s="1" t="inlineStr">
         <is>
-          <t>6x1km</t>
+          <t>Long Run</t>
         </is>
       </c>
       <c r="C170" s="1" t="inlineStr">
@@ -5301,7 +5297,7 @@
       </c>
       <c r="B171" s="1" t="inlineStr">
         <is>
-          <t>1km Repeat Intervals</t>
+          <t>6x1km</t>
         </is>
       </c>
       <c r="C171" s="1" t="inlineStr">
@@ -5333,7 +5329,7 @@
       </c>
       <c r="B172" s="1" t="inlineStr">
         <is>
-          <t>4x4 VO2</t>
+          <t>1km Repeat Intervals</t>
         </is>
       </c>
       <c r="C172" s="1" t="inlineStr">
@@ -5365,7 +5361,7 @@
       </c>
       <c r="B173" s="1" t="inlineStr">
         <is>
-          <t>200m/400m Repeat Runs</t>
+          <t>4x4 VO2</t>
         </is>
       </c>
       <c r="C173" s="1" t="inlineStr">
@@ -5380,12 +5376,12 @@
       </c>
       <c r="E173" s="1" t="inlineStr">
         <is>
-          <t>1+ years</t>
+          <t>everyone</t>
         </is>
       </c>
       <c r="F173" s="1" t="inlineStr">
         <is>
-          <t>⚑ sprint-adjacent speed endurance at high impact — the training-age ladder is a rough fit for a session format.</t>
+          <t>session format, not an individual movement — no meaningful muscle group.</t>
         </is>
       </c>
     </row>
@@ -5397,7 +5393,7 @@
       </c>
       <c r="B174" s="1" t="inlineStr">
         <is>
-          <t>Footy Fartlek</t>
+          <t>200m/400m Repeat Runs</t>
         </is>
       </c>
       <c r="C174" s="1" t="inlineStr">
@@ -5412,12 +5408,12 @@
       </c>
       <c r="E174" s="1" t="inlineStr">
         <is>
-          <t>everyone</t>
+          <t>1+ years</t>
         </is>
       </c>
       <c r="F174" s="1" t="inlineStr">
         <is>
-          <t>session format, not an individual movement — no meaningful muscle group.</t>
+          <t>⚑ sprint-adjacent speed endurance at high impact — the training-age ladder is a rough fit for a session format.</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5425,7 @@
       </c>
       <c r="B175" s="1" t="inlineStr">
         <is>
-          <t>Hard Row Intervals</t>
+          <t>Footy Fartlek</t>
         </is>
       </c>
       <c r="C175" s="1" t="inlineStr">
@@ -5461,7 +5457,7 @@
       </c>
       <c r="B176" s="1" t="inlineStr">
         <is>
-          <t>Hard SkiErg Intervals</t>
+          <t>Hard Row Intervals</t>
         </is>
       </c>
       <c r="C176" s="1" t="inlineStr">
@@ -5493,7 +5489,7 @@
       </c>
       <c r="B177" s="1" t="inlineStr">
         <is>
-          <t>Hard Assault Bike Intervals</t>
+          <t>Hard SkiErg Intervals</t>
         </is>
       </c>
       <c r="C177" s="1" t="inlineStr">
@@ -5525,7 +5521,7 @@
       </c>
       <c r="B178" s="1" t="inlineStr">
         <is>
-          <t>Erg EMOM</t>
+          <t>Hard Assault Bike Intervals</t>
         </is>
       </c>
       <c r="C178" s="1" t="inlineStr">
@@ -5557,7 +5553,7 @@
       </c>
       <c r="B179" s="1" t="inlineStr">
         <is>
-          <t>Tempo Run</t>
+          <t>Erg EMOM</t>
         </is>
       </c>
       <c r="C179" s="1" t="inlineStr">
@@ -5589,7 +5585,7 @@
       </c>
       <c r="B180" s="1" t="inlineStr">
         <is>
-          <t>Long Nasal Run</t>
+          <t>Tempo Run</t>
         </is>
       </c>
       <c r="C180" s="1" t="inlineStr">
@@ -5621,7 +5617,7 @@
       </c>
       <c r="B181" s="1" t="inlineStr">
         <is>
-          <t>30:30 Tempo Blocks</t>
+          <t>Long Nasal Run</t>
         </is>
       </c>
       <c r="C181" s="1" t="inlineStr">
@@ -5653,7 +5649,7 @@
       </c>
       <c r="B182" s="1" t="inlineStr">
         <is>
-          <t>Tempo Intervals (1min on / 1min easy)</t>
+          <t>30:30 Tempo Blocks</t>
         </is>
       </c>
       <c r="C182" s="1" t="inlineStr">
@@ -5685,7 +5681,7 @@
       </c>
       <c r="B183" s="1" t="inlineStr">
         <is>
-          <t>Cruise Intervals</t>
+          <t>Tempo Intervals (1min on / 1min easy)</t>
         </is>
       </c>
       <c r="C183" s="1" t="inlineStr">
@@ -5717,7 +5713,7 @@
       </c>
       <c r="B184" s="1" t="inlineStr">
         <is>
-          <t>Bike/Row/Ski Tempo Intervals</t>
+          <t>Cruise Intervals</t>
         </is>
       </c>
       <c r="C184" s="1" t="inlineStr">
@@ -5749,7 +5745,7 @@
       </c>
       <c r="B185" s="1" t="inlineStr">
         <is>
-          <t>Air Bike Sprints</t>
+          <t>Bike/Row/Ski Tempo Intervals</t>
         </is>
       </c>
       <c r="C185" s="1" t="inlineStr">
@@ -5781,7 +5777,7 @@
       </c>
       <c r="B186" s="1" t="inlineStr">
         <is>
-          <t>Row Intervals</t>
+          <t>Air Bike Sprints</t>
         </is>
       </c>
       <c r="C186" s="1" t="inlineStr">
@@ -5813,7 +5809,7 @@
       </c>
       <c r="B187" s="1" t="inlineStr">
         <is>
-          <t>SkiErg Intervals</t>
+          <t>Row Intervals</t>
         </is>
       </c>
       <c r="C187" s="1" t="inlineStr">
@@ -5845,7 +5841,7 @@
       </c>
       <c r="B188" s="1" t="inlineStr">
         <is>
-          <t>Assault Bike Intervals</t>
+          <t>SkiErg Intervals</t>
         </is>
       </c>
       <c r="C188" s="1" t="inlineStr">
@@ -5877,7 +5873,7 @@
       </c>
       <c r="B189" s="1" t="inlineStr">
         <is>
-          <t>Flush Run</t>
+          <t>Assault Bike Intervals</t>
         </is>
       </c>
       <c r="C189" s="1" t="inlineStr">
@@ -5909,7 +5905,7 @@
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>Easy Bike</t>
+          <t>Flush Run</t>
         </is>
       </c>
       <c r="C190" s="1" t="inlineStr">
@@ -5941,7 +5937,7 @@
       </c>
       <c r="B191" s="1" t="inlineStr">
         <is>
-          <t>Easy Row</t>
+          <t>Easy Bike</t>
         </is>
       </c>
       <c r="C191" s="1" t="inlineStr">
@@ -5973,7 +5969,7 @@
       </c>
       <c r="B192" s="1" t="inlineStr">
         <is>
-          <t>Easy Ski</t>
+          <t>Easy Row</t>
         </is>
       </c>
       <c r="C192" s="1" t="inlineStr">
@@ -6005,7 +6001,7 @@
       </c>
       <c r="B193" s="1" t="inlineStr">
         <is>
-          <t>Easy Swim</t>
+          <t>Easy Ski</t>
         </is>
       </c>
       <c r="C193" s="1" t="inlineStr">
@@ -6037,59 +6033,63 @@
       </c>
       <c r="B194" s="1" t="inlineStr">
         <is>
+          <t>Easy Swim</t>
+        </is>
+      </c>
+      <c r="C194" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D194" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E194" s="1" t="inlineStr">
+        <is>
+          <t>everyone</t>
+        </is>
+      </c>
+      <c r="F194" s="1" t="inlineStr">
+        <is>
+          <t>session format, not an individual movement — no meaningful muscle group.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="1" t="inlineStr">
+        <is>
+          <t>Conditioning</t>
+        </is>
+      </c>
+      <c r="B195" s="1" t="inlineStr">
+        <is>
           <t>Light Circuits</t>
         </is>
       </c>
-      <c r="C194" s="1" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D194" s="1" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E194" s="1" t="inlineStr">
-        <is>
-          <t>everyone</t>
-        </is>
-      </c>
-      <c r="F194" s="1" t="inlineStr">
+      <c r="C195" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D195" s="1" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E195" s="1" t="inlineStr">
+        <is>
+          <t>everyone</t>
+        </is>
+      </c>
+      <c r="F195" s="1" t="inlineStr">
         <is>
           <t>session format, not an individual movement — no meaningful muscle group.</t>
         </is>
       </c>
     </row>
-    <row r="195"/>
-    <row r="196">
-      <c r="A196" s="1" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="B196" s="1" t="inlineStr">
-        <is>
-          <t>Vertical Jump</t>
-        </is>
-      </c>
-      <c r="C196" s="1" t="inlineStr">
-        <is>
-          <t>Glutes, Quads, Calves</t>
-        </is>
-      </c>
-      <c r="D196" s="1" t="inlineStr">
-        <is>
-          <t>Hamstrings, Midline</t>
-        </is>
-      </c>
-      <c r="E196" s="1" t="inlineStr">
-        <is>
-          <t>everyone</t>
-        </is>
-      </c>
-      <c r="F196" s="1" t="inlineStr"/>
-    </row>
+    <row r="196"/>
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
@@ -6098,17 +6098,17 @@
       </c>
       <c r="B197" s="1" t="inlineStr">
         <is>
-          <t>Pogo Hops</t>
+          <t>Vertical Jump</t>
         </is>
       </c>
       <c r="C197" s="1" t="inlineStr">
         <is>
-          <t>Calves</t>
+          <t>Glutes, Quads, Calves</t>
         </is>
       </c>
       <c r="D197" s="1" t="inlineStr">
         <is>
-          <t>Quads, Midline</t>
+          <t>Hamstrings, Midline</t>
         </is>
       </c>
       <c r="E197" s="1" t="inlineStr">
@@ -6116,11 +6116,7 @@
           <t>everyone</t>
         </is>
       </c>
-      <c r="F197" s="1" t="inlineStr">
-        <is>
-          <t>takes over when lower niggle (your spec)</t>
-        </is>
-      </c>
+      <c r="F197" s="1" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
@@ -6130,17 +6126,17 @@
       </c>
       <c r="B198" s="1" t="inlineStr">
         <is>
-          <t>Lateral Jump</t>
+          <t>Pogo Hops</t>
         </is>
       </c>
       <c r="C198" s="1" t="inlineStr">
         <is>
-          <t>Glutes, Outer hip</t>
+          <t>Calves</t>
         </is>
       </c>
       <c r="D198" s="1" t="inlineStr">
         <is>
-          <t>Quads, Calves, Midline</t>
+          <t>Quads, Midline</t>
         </is>
       </c>
       <c r="E198" s="1" t="inlineStr">
@@ -6150,7 +6146,7 @@
       </c>
       <c r="F198" s="1" t="inlineStr">
         <is>
-          <t>your spec: beginner friendly</t>
+          <t>takes over when lower niggle (your spec)</t>
         </is>
       </c>
     </row>
@@ -6162,27 +6158,27 @@
       </c>
       <c r="B199" s="1" t="inlineStr">
         <is>
-          <t>Kneeling Jump</t>
+          <t>Lateral Jump</t>
         </is>
       </c>
       <c r="C199" s="1" t="inlineStr">
         <is>
-          <t>Glutes, Quads</t>
+          <t>Glutes, Outer hip</t>
         </is>
       </c>
       <c r="D199" s="1" t="inlineStr">
         <is>
-          <t>Hamstrings, Midline</t>
+          <t>Quads, Calves, Midline</t>
         </is>
       </c>
       <c r="E199" s="1" t="inlineStr">
         <is>
-          <t>2+ years</t>
+          <t>everyone</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr">
         <is>
-          <t>your spec: consistent+</t>
+          <t>your spec: beginner friendly</t>
         </is>
       </c>
     </row>
@@ -6194,17 +6190,17 @@
       </c>
       <c r="B200" s="1" t="inlineStr">
         <is>
-          <t>RFE Split Squat Jump</t>
+          <t>Kneeling Jump</t>
         </is>
       </c>
       <c r="C200" s="1" t="inlineStr">
         <is>
-          <t>Quads, Glutes</t>
+          <t>Glutes, Quads</t>
         </is>
       </c>
       <c r="D200" s="1" t="inlineStr">
         <is>
-          <t>Hamstrings, Calves, Midline</t>
+          <t>Hamstrings, Midline</t>
         </is>
       </c>
       <c r="E200" s="1" t="inlineStr">
@@ -6212,9 +6208,9 @@
           <t>2+ years</t>
         </is>
       </c>
-      <c r="F200" s="3" t="inlineStr">
-        <is>
-          <t>FLAG — gate proposed, confirm</t>
+      <c r="F200" s="1" t="inlineStr">
+        <is>
+          <t>your spec: consistent+</t>
         </is>
       </c>
     </row>
@@ -6226,25 +6222,29 @@
       </c>
       <c r="B201" s="1" t="inlineStr">
         <is>
-          <t>Explosive Push-up</t>
+          <t>RFE Split Squat Jump</t>
         </is>
       </c>
       <c r="C201" s="1" t="inlineStr">
         <is>
-          <t>Chest, Triceps</t>
+          <t>Quads, Glutes</t>
         </is>
       </c>
       <c r="D201" s="1" t="inlineStr">
         <is>
-          <t>Shoulders, Midline</t>
+          <t>Hamstrings, Calves, Midline</t>
         </is>
       </c>
       <c r="E201" s="1" t="inlineStr">
         <is>
-          <t>everyone</t>
-        </is>
-      </c>
-      <c r="F201" s="1" t="inlineStr"/>
+          <t>2+ years</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr">
+        <is>
+          <t>FLAG — gate proposed, confirm</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="B202" s="1" t="inlineStr">
         <is>
-          <t>Speed Bench</t>
+          <t>Explosive Push-up</t>
         </is>
       </c>
       <c r="C202" s="1" t="inlineStr">
@@ -6264,19 +6264,15 @@
       </c>
       <c r="D202" s="1" t="inlineStr">
         <is>
-          <t>Shoulders, Lats</t>
+          <t>Shoulders, Midline</t>
         </is>
       </c>
       <c r="E202" s="1" t="inlineStr">
         <is>
-          <t>2+ years</t>
-        </is>
-      </c>
-      <c r="F202" s="3" t="inlineStr">
-        <is>
-          <t>FLAG — gate proposed, confirm</t>
-        </is>
-      </c>
+          <t>everyone</t>
+        </is>
+      </c>
+      <c r="F202" s="1" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
@@ -6286,25 +6282,57 @@
       </c>
       <c r="B203" s="1" t="inlineStr">
         <is>
+          <t>Speed Bench</t>
+        </is>
+      </c>
+      <c r="C203" s="1" t="inlineStr">
+        <is>
+          <t>Chest, Triceps</t>
+        </is>
+      </c>
+      <c r="D203" s="1" t="inlineStr">
+        <is>
+          <t>Shoulders, Lats</t>
+        </is>
+      </c>
+      <c r="E203" s="1" t="inlineStr">
+        <is>
+          <t>2+ years</t>
+        </is>
+      </c>
+      <c r="F203" s="3" t="inlineStr">
+        <is>
+          <t>FLAG — gate proposed, confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="B204" s="1" t="inlineStr">
+        <is>
           <t>Speed Trap Bar Deadlift</t>
         </is>
       </c>
-      <c r="C203" s="1" t="inlineStr">
+      <c r="C204" s="1" t="inlineStr">
         <is>
           <t>Glutes, Hamstrings</t>
         </is>
       </c>
-      <c r="D203" s="1" t="inlineStr">
+      <c r="D204" s="1" t="inlineStr">
         <is>
           <t>Quads, Upper back, Grip</t>
         </is>
       </c>
-      <c r="E203" s="1" t="inlineStr">
+      <c r="E204" s="1" t="inlineStr">
         <is>
           <t>2+ years</t>
         </is>
       </c>
-      <c r="F203" s="3" t="inlineStr">
+      <c r="F204" s="3" t="inlineStr">
         <is>
           <t>FLAG — gate proposed, confirm</t>
         </is>

</xml_diff>